<commit_message>
test: Add comprehensive Right Panel data tests
Add test cases for Right Panel (K14-U31) with:
- Complete data: 18 rows with dates (L14-L31), amounts in EUR (M14-M31)
  and local currency (N14-N31)
- Realistic data: Invoice numbers (RGG-101..118, INV-201..218),
  variable dates (March-April 2024), amounts 250-1300 EUR

Tests verify all fields are populated correctly through the API:
- LeftNumber, LeftDate, LeftAmount1, LeftAmount2 (K-N)
- RightNumber, RightDate, RightAmount1, RightAmount2 (R-U)

Generated test files:
- right_panel_complete_data.xlsx (sequential data)
- right_panel_realistic_data.xlsx (realistic invoice data)
- test_right_panel_complete.xlsx (example output)
</commit_message>
<xml_diff>
--- a/src/v2/tests/formula_eval_test.xlsx
+++ b/src/v2/tests/formula_eval_test.xlsx
@@ -2051,57 +2051,57 @@
     <xf numFmtId="167" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -2424,12 +2424,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:22">
-      <c r="B1" s="56" t="str">
+      <c r="B1" s="52" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,2,FALSE))</f>
         <v>F I N A N Z B E R I C H T</v>
       </c>
       <c r="C1" s="2"/>
-      <c r="J1" s="52" t="str">
+      <c r="J1" s="58" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,60,FALSE))</f>
         <v>Tipp:</v>
       </c>
@@ -2444,14 +2444,14 @@
         <v>0</v>
       </c>
       <c r="C2" s="3"/>
-      <c r="D2" s="48" t="str">
+      <c r="D2" s="63" t="str">
         <f>IF($E$2="","Chose your language",VLOOKUP($E$2,Sprachversionen!$B:$BN,27,FALSE))</f>
         <v>Sprache</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="58" t="str">
+      <c r="J2" s="67" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,61,FALSE))</f>
         <v>Bitte nutzen Sie zum ausfüllen des Finanzberichts unsere Ausfüllhilfe auf unserer Webseite:</v>
       </c>
@@ -2462,12 +2462,12 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3" spans="2:22">
-      <c r="B3" s="56" t="str">
+      <c r="B3" s="52" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,3,FALSE))</f>
         <v>ÜBERSICHT ÜBER EINNAHMEN UND AUSGABEN</v>
       </c>
       <c r="C3" s="2"/>
-      <c r="D3" s="48" t="str">
+      <c r="D3" s="63" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE))</f>
         <v>Lokalwährung</v>
       </c>
@@ -2482,7 +2482,7 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4" spans="2:22" ht="12" customHeight="1">
-      <c r="J4" s="62" t="str">
+      <c r="J4" s="61" t="str">
         <f>HYPERLINK(VLOOKUP($E$2,Sprachversionen!$B:$BN,62,FALSE))</f>
         <v>https://www.kindermissionswerk.org/fuer-partner/service</v>
       </c>
@@ -2493,7 +2493,7 @@
       <c r="O4" s="5"/>
     </row>
     <row r="5" spans="2:22">
-      <c r="B5" s="48" t="str">
+      <c r="B5" s="63" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,4,FALSE))</f>
         <v>Projektnummer</v>
       </c>
@@ -2503,7 +2503,7 @@
       </c>
     </row>
     <row r="6" spans="2:22">
-      <c r="B6" s="48" t="str">
+      <c r="B6" s="63" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,26,FALSE))</f>
         <v>Projekttitel</v>
       </c>
@@ -2527,17 +2527,17 @@
       <c r="J7" s="13"/>
     </row>
     <row r="8" spans="2:22">
-      <c r="B8" s="48" t="str">
+      <c r="B8" s="63" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,5,FALSE))</f>
         <v>Projektlaufzeit</v>
       </c>
       <c r="C8" s="6"/>
-      <c r="D8" s="53" t="str">
+      <c r="D8" s="55" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,7,FALSE))</f>
         <v>von (TT MM JJJJ):</v>
       </c>
       <c r="E8" s="8"/>
-      <c r="F8" s="53" t="str">
+      <c r="F8" s="55" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,8,FALSE))</f>
         <v>bis (TT MM JJJJ):</v>
       </c>
@@ -2550,17 +2550,17 @@
       </c>
     </row>
     <row r="9" spans="2:22">
-      <c r="B9" s="48" t="str">
+      <c r="B9" s="63" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,6,FALSE))</f>
         <v>Aktueller Berichtszeitraum</v>
       </c>
       <c r="C9" s="6"/>
-      <c r="D9" s="53" t="str">
+      <c r="D9" s="55" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,7,FALSE))</f>
         <v>von (TT MM JJJJ):</v>
       </c>
       <c r="E9" s="8"/>
-      <c r="F9" s="53" t="str">
+      <c r="F9" s="55" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,8,FALSE))</f>
         <v>bis (TT MM JJJJ):</v>
       </c>
@@ -2572,7 +2572,7 @@
     <row r="11" spans="2:22" ht="12.75" customHeight="1">
       <c r="B11" s="16"/>
       <c r="C11" s="26"/>
-      <c r="D11" s="57" t="str">
+      <c r="D11" s="48" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,11,FALSE))</f>
         <v>Bewilligtes Budget</v>
       </c>
@@ -2580,11 +2580,11 @@
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,12,FALSE))</f>
         <v>Einnahmen im Berichtszeitraum</v>
       </c>
-      <c r="F11" s="57" t="str">
+      <c r="F11" s="48" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,13,FALSE))</f>
         <v>Einnahmen der gesamten Projektlaufzeit</v>
       </c>
-      <c r="G11" s="57" t="str">
+      <c r="G11" s="48" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,14,FALSE))</f>
         <v>% erhaltene Einnahmen</v>
       </c>
@@ -2592,7 +2592,7 @@
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,15,FALSE))</f>
         <v>Begründung der Budgetüber- oder unterschreitung</v>
       </c>
-      <c r="J11" s="65" t="str">
+      <c r="J11" s="59" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>KMW Mittel*</v>
       </c>
@@ -2601,7 +2601,7 @@
       <c r="M11" s="34"/>
       <c r="N11" s="34"/>
       <c r="O11" s="35"/>
-      <c r="Q11" s="65" t="str">
+      <c r="Q11" s="59" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>KMW Mittel*</v>
       </c>
@@ -2612,7 +2612,7 @@
       <c r="V11" s="35"/>
     </row>
     <row r="12" spans="2:22">
-      <c r="B12" s="67" t="str">
+      <c r="B12" s="64" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,9,FALSE))</f>
         <v>EINNAHMEN</v>
       </c>
@@ -2636,7 +2636,7 @@
       <c r="V12" s="37"/>
     </row>
     <row r="13" spans="2:22">
-      <c r="B13" s="54" t="str">
+      <c r="B13" s="62" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,10,FALSE))</f>
         <v>(in lokaler Währung)</v>
       </c>
@@ -2648,37 +2648,37 @@
       <c r="H13" s="19"/>
       <c r="J13" s="36"/>
       <c r="K13" s="1"/>
-      <c r="L13" s="49" t="str">
+      <c r="L13" s="50" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,22,FALSE))</f>
         <v>Datum</v>
       </c>
-      <c r="M13" s="49" t="str">
+      <c r="M13" s="50" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,63,FALSE))</f>
         <v>Euro</v>
       </c>
-      <c r="N13" s="49" t="str">
+      <c r="N13" s="50" t="str">
         <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>EUR</v>
       </c>
-      <c r="O13" s="59" t="str">
+      <c r="O13" s="53" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE))</f>
         <v>WK</v>
       </c>
       <c r="Q13" s="36"/>
       <c r="R13" s="1"/>
-      <c r="S13" s="49" t="str">
+      <c r="S13" s="50" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,22,FALSE))</f>
         <v>Datum</v>
       </c>
-      <c r="T13" s="49" t="str">
+      <c r="T13" s="50" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,63,FALSE))</f>
         <v>Euro</v>
       </c>
-      <c r="U13" s="49" t="str">
+      <c r="U13" s="50" t="str">
         <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>EUR</v>
       </c>
-      <c r="V13" s="59" t="str">
+      <c r="V13" s="53" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE))</f>
         <v>WK</v>
       </c>
@@ -2721,7 +2721,7 @@
       </c>
     </row>
     <row r="15" spans="2:22">
-      <c r="B15" s="64" t="str">
+      <c r="B15" s="60" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,16,FALSE))</f>
         <v>Saldovortrag (aus vorherigem Berichtszeitraum)</v>
       </c>
@@ -2767,7 +2767,7 @@
       </c>
     </row>
     <row r="16" spans="2:22">
-      <c r="B16" s="55" t="str">
+      <c r="B16" s="56" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,17,FALSE))</f>
         <v>Lokale Eigenleistung</v>
       </c>
@@ -2781,7 +2781,7 @@
       <c r="F16" s="28">
         <v>1000</v>
       </c>
-      <c r="G16" s="50">
+      <c r="G16" s="49">
         <f>IFERROR(F16/D16,0)</f>
         <v>0.5</v>
       </c>
@@ -2816,7 +2816,7 @@
       </c>
     </row>
     <row r="17" spans="2:22">
-      <c r="B17" s="55" t="str">
+      <c r="B17" s="56" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,18,FALSE))</f>
         <v>Beiträge von dritter Seite</v>
       </c>
@@ -2830,7 +2830,7 @@
       <c r="F17" s="28">
         <v>1500</v>
       </c>
-      <c r="G17" s="50">
+      <c r="G17" s="49">
         <f>IFERROR(F17/D17,0)</f>
         <v>0.5</v>
       </c>
@@ -2865,7 +2865,7 @@
       </c>
     </row>
     <row r="18" spans="2:22">
-      <c r="B18" s="55" t="str">
+      <c r="B18" s="56" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>KMW Mittel*</v>
       </c>
@@ -2879,7 +2879,7 @@
       <c r="F18" s="28">
         <v>2000</v>
       </c>
-      <c r="G18" s="50">
+      <c r="G18" s="49">
         <f>IFERROR(F18/D18,0)</f>
         <v>0.5</v>
       </c>
@@ -2914,7 +2914,7 @@
       </c>
     </row>
     <row r="19" spans="2:22">
-      <c r="B19" s="55" t="str">
+      <c r="B19" s="56" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,20,FALSE))</f>
         <v>Zinserträge</v>
       </c>
@@ -2928,7 +2928,7 @@
       <c r="F19" s="28">
         <v>2500</v>
       </c>
-      <c r="G19" s="50">
+      <c r="G19" s="49">
         <f>IFERROR(F19/D19,0)</f>
         <v>0.5</v>
       </c>
@@ -2963,24 +2963,24 @@
       </c>
     </row>
     <row r="20" spans="2:22">
-      <c r="B20" s="63" t="str">
+      <c r="B20" s="57" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,21,FALSE))</f>
         <v>GESAMT</v>
       </c>
       <c r="C20" s="25"/>
-      <c r="D20" s="60">
+      <c r="D20" s="54">
         <f>SUMPRODUCT(ROUND(D15:D19,2))</f>
         <v>15000</v>
       </c>
-      <c r="E20" s="60">
+      <c r="E20" s="54">
         <f>SUMPRODUCT(ROUND(E15:E19,2))</f>
         <v>1500</v>
       </c>
-      <c r="F20" s="60">
+      <c r="F20" s="54">
         <f>SUMPRODUCT(ROUND(F15:F19,2))</f>
         <v>7500</v>
       </c>
-      <c r="G20" s="61">
+      <c r="G20" s="65">
         <f>IFERROR(F20/D20,0)</f>
         <v>0.5</v>
       </c>

</xml_diff>

<commit_message>
fix: Remove J7/J8/J9 and K/R columns from API (they are formulas)
API fields corrected to only include actual input cells:
- E2:E3 (Language, Currency)
- D5, D6 (Project Number, Title)
- E8:E9, G8:G9 (Project dates, Report dates)
- D15:F19 (Budget, Income Report Period, Income Total)
- H15:H19 (Reason)
- L14:N31 (Date, Euro, Local - left side)
- S14:U31 (Date, Euro, Local - right side)

Removed from API (these are formulas in Excel):
- J7, J8 (Exchange rate date/value - formulas!)
- J9 (User input in Excel, not via API)
- K14:K31 (Number left - formulas!)
- R14:R31 (Number right - formulas!)
- G15:G19 (Percent - IFERROR division formulas)
</commit_message>
<xml_diff>
--- a/src/v2/tests/formula_eval_test.xlsx
+++ b/src/v2/tests/formula_eval_test.xlsx
@@ -2051,57 +2051,57 @@
     <xf numFmtId="167" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -2424,12 +2424,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:22">
-      <c r="B1" s="52" t="str">
+      <c r="B1" s="66" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,2,FALSE))</f>
         <v>F I N A N Z B E R I C H T</v>
       </c>
       <c r="C1" s="2"/>
-      <c r="J1" s="58" t="str">
+      <c r="J1" s="60" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,60,FALSE))</f>
         <v>Tipp:</v>
       </c>
@@ -2444,14 +2444,14 @@
         <v>0</v>
       </c>
       <c r="C2" s="3"/>
-      <c r="D2" s="63" t="str">
+      <c r="D2" s="49" t="str">
         <f>IF($E$2="","Chose your language",VLOOKUP($E$2,Sprachversionen!$B:$BN,27,FALSE))</f>
         <v>Sprache</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="67" t="str">
+      <c r="J2" s="51" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,61,FALSE))</f>
         <v>Bitte nutzen Sie zum ausfüllen des Finanzberichts unsere Ausfüllhilfe auf unserer Webseite:</v>
       </c>
@@ -2462,12 +2462,12 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3" spans="2:22">
-      <c r="B3" s="52" t="str">
+      <c r="B3" s="66" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,3,FALSE))</f>
         <v>ÜBERSICHT ÜBER EINNAHMEN UND AUSGABEN</v>
       </c>
       <c r="C3" s="2"/>
-      <c r="D3" s="63" t="str">
+      <c r="D3" s="49" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE))</f>
         <v>Lokalwährung</v>
       </c>
@@ -2482,7 +2482,7 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4" spans="2:22" ht="12" customHeight="1">
-      <c r="J4" s="61" t="str">
+      <c r="J4" s="62" t="str">
         <f>HYPERLINK(VLOOKUP($E$2,Sprachversionen!$B:$BN,62,FALSE))</f>
         <v>https://www.kindermissionswerk.org/fuer-partner/service</v>
       </c>
@@ -2493,7 +2493,7 @@
       <c r="O4" s="5"/>
     </row>
     <row r="5" spans="2:22">
-      <c r="B5" s="63" t="str">
+      <c r="B5" s="49" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,4,FALSE))</f>
         <v>Projektnummer</v>
       </c>
@@ -2503,7 +2503,7 @@
       </c>
     </row>
     <row r="6" spans="2:22">
-      <c r="B6" s="63" t="str">
+      <c r="B6" s="49" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,26,FALSE))</f>
         <v>Projekttitel</v>
       </c>
@@ -2527,17 +2527,17 @@
       <c r="J7" s="13"/>
     </row>
     <row r="8" spans="2:22">
-      <c r="B8" s="63" t="str">
+      <c r="B8" s="49" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,5,FALSE))</f>
         <v>Projektlaufzeit</v>
       </c>
       <c r="C8" s="6"/>
-      <c r="D8" s="55" t="str">
+      <c r="D8" s="54" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,7,FALSE))</f>
         <v>von (TT MM JJJJ):</v>
       </c>
       <c r="E8" s="8"/>
-      <c r="F8" s="55" t="str">
+      <c r="F8" s="54" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,8,FALSE))</f>
         <v>bis (TT MM JJJJ):</v>
       </c>
@@ -2550,17 +2550,17 @@
       </c>
     </row>
     <row r="9" spans="2:22">
-      <c r="B9" s="63" t="str">
+      <c r="B9" s="49" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,6,FALSE))</f>
         <v>Aktueller Berichtszeitraum</v>
       </c>
       <c r="C9" s="6"/>
-      <c r="D9" s="55" t="str">
+      <c r="D9" s="54" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,7,FALSE))</f>
         <v>von (TT MM JJJJ):</v>
       </c>
       <c r="E9" s="8"/>
-      <c r="F9" s="55" t="str">
+      <c r="F9" s="54" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,8,FALSE))</f>
         <v>bis (TT MM JJJJ):</v>
       </c>
@@ -2572,23 +2572,23 @@
     <row r="11" spans="2:22" ht="12.75" customHeight="1">
       <c r="B11" s="16"/>
       <c r="C11" s="26"/>
-      <c r="D11" s="48" t="str">
+      <c r="D11" s="55" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,11,FALSE))</f>
         <v>Bewilligtes Budget</v>
       </c>
-      <c r="E11" s="51" t="str">
+      <c r="E11" s="63" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,12,FALSE))</f>
         <v>Einnahmen im Berichtszeitraum</v>
       </c>
-      <c r="F11" s="48" t="str">
+      <c r="F11" s="55" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,13,FALSE))</f>
         <v>Einnahmen der gesamten Projektlaufzeit</v>
       </c>
-      <c r="G11" s="48" t="str">
+      <c r="G11" s="55" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,14,FALSE))</f>
         <v>% erhaltene Einnahmen</v>
       </c>
-      <c r="H11" s="66" t="str">
+      <c r="H11" s="67" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,15,FALSE))</f>
         <v>Begründung der Budgetüber- oder unterschreitung</v>
       </c>
@@ -2636,7 +2636,7 @@
       <c r="V12" s="37"/>
     </row>
     <row r="13" spans="2:22">
-      <c r="B13" s="62" t="str">
+      <c r="B13" s="56" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,10,FALSE))</f>
         <v>(in lokaler Währung)</v>
       </c>
@@ -2648,37 +2648,37 @@
       <c r="H13" s="19"/>
       <c r="J13" s="36"/>
       <c r="K13" s="1"/>
-      <c r="L13" s="50" t="str">
+      <c r="L13" s="48" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,22,FALSE))</f>
         <v>Datum</v>
       </c>
-      <c r="M13" s="50" t="str">
+      <c r="M13" s="48" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,63,FALSE))</f>
         <v>Euro</v>
       </c>
-      <c r="N13" s="50" t="str">
+      <c r="N13" s="48" t="str">
         <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>EUR</v>
       </c>
-      <c r="O13" s="53" t="str">
+      <c r="O13" s="57" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE))</f>
         <v>WK</v>
       </c>
       <c r="Q13" s="36"/>
       <c r="R13" s="1"/>
-      <c r="S13" s="50" t="str">
+      <c r="S13" s="48" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,22,FALSE))</f>
         <v>Datum</v>
       </c>
-      <c r="T13" s="50" t="str">
+      <c r="T13" s="48" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,63,FALSE))</f>
         <v>Euro</v>
       </c>
-      <c r="U13" s="50" t="str">
+      <c r="U13" s="48" t="str">
         <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>EUR</v>
       </c>
-      <c r="V13" s="53" t="str">
+      <c r="V13" s="57" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE))</f>
         <v>WK</v>
       </c>
@@ -2721,7 +2721,7 @@
       </c>
     </row>
     <row r="15" spans="2:22">
-      <c r="B15" s="60" t="str">
+      <c r="B15" s="65" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,16,FALSE))</f>
         <v>Saldovortrag (aus vorherigem Berichtszeitraum)</v>
       </c>
@@ -2767,7 +2767,7 @@
       </c>
     </row>
     <row r="16" spans="2:22">
-      <c r="B16" s="56" t="str">
+      <c r="B16" s="50" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,17,FALSE))</f>
         <v>Lokale Eigenleistung</v>
       </c>
@@ -2781,7 +2781,7 @@
       <c r="F16" s="28">
         <v>1000</v>
       </c>
-      <c r="G16" s="49">
+      <c r="G16" s="52">
         <f>IFERROR(F16/D16,0)</f>
         <v>0.5</v>
       </c>
@@ -2816,7 +2816,7 @@
       </c>
     </row>
     <row r="17" spans="2:22">
-      <c r="B17" s="56" t="str">
+      <c r="B17" s="50" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,18,FALSE))</f>
         <v>Beiträge von dritter Seite</v>
       </c>
@@ -2830,7 +2830,7 @@
       <c r="F17" s="28">
         <v>1500</v>
       </c>
-      <c r="G17" s="49">
+      <c r="G17" s="52">
         <f>IFERROR(F17/D17,0)</f>
         <v>0.5</v>
       </c>
@@ -2865,7 +2865,7 @@
       </c>
     </row>
     <row r="18" spans="2:22">
-      <c r="B18" s="56" t="str">
+      <c r="B18" s="50" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>KMW Mittel*</v>
       </c>
@@ -2879,7 +2879,7 @@
       <c r="F18" s="28">
         <v>2000</v>
       </c>
-      <c r="G18" s="49">
+      <c r="G18" s="52">
         <f>IFERROR(F18/D18,0)</f>
         <v>0.5</v>
       </c>
@@ -2914,7 +2914,7 @@
       </c>
     </row>
     <row r="19" spans="2:22">
-      <c r="B19" s="56" t="str">
+      <c r="B19" s="50" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,20,FALSE))</f>
         <v>Zinserträge</v>
       </c>
@@ -2928,7 +2928,7 @@
       <c r="F19" s="28">
         <v>2500</v>
       </c>
-      <c r="G19" s="49">
+      <c r="G19" s="52">
         <f>IFERROR(F19/D19,0)</f>
         <v>0.5</v>
       </c>
@@ -2963,24 +2963,24 @@
       </c>
     </row>
     <row r="20" spans="2:22">
-      <c r="B20" s="57" t="str">
+      <c r="B20" s="61" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,21,FALSE))</f>
         <v>GESAMT</v>
       </c>
       <c r="C20" s="25"/>
-      <c r="D20" s="54">
+      <c r="D20" s="58">
         <f>SUMPRODUCT(ROUND(D15:D19,2))</f>
         <v>15000</v>
       </c>
-      <c r="E20" s="54">
+      <c r="E20" s="58">
         <f>SUMPRODUCT(ROUND(E15:E19,2))</f>
         <v>1500</v>
       </c>
-      <c r="F20" s="54">
+      <c r="F20" s="58">
         <f>SUMPRODUCT(ROUND(F15:F19,2))</f>
         <v>7500</v>
       </c>
-      <c r="G20" s="65">
+      <c r="G20" s="53">
         <f>IFERROR(F20/D20,0)</f>
         <v>0.5</v>
       </c>

</xml_diff>

<commit_message>
fix: Completely remove J7/J8/J9 exchange rate cells from API
- Removed ExchangeRateDate, ExchangeRateValue, ExchangeRateInput from HeaderInputCell enum
- Removed J7, J8, J9 address constants from registry
- Removed exchange_rate() getter and with_exchange_rate() setter from ReportValues
- Updated documentation to clarify J7/J8/J9 are NOT API input fields
- All 26 tests pass

These cells are formulas/user inputs in Excel, not API input fields.
</commit_message>
<xml_diff>
--- a/src/v2/tests/formula_eval_test.xlsx
+++ b/src/v2/tests/formula_eval_test.xlsx
@@ -2057,51 +2057,51 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -2424,12 +2424,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:22">
-      <c r="B1" s="66" t="str">
+      <c r="B1" s="52" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,2,FALSE))</f>
         <v>F I N A N Z B E R I C H T</v>
       </c>
       <c r="C1" s="2"/>
-      <c r="J1" s="60" t="str">
+      <c r="J1" s="61" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,60,FALSE))</f>
         <v>Tipp:</v>
       </c>
@@ -2451,7 +2451,7 @@
       <c r="E2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="51" t="str">
+      <c r="J2" s="67" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,61,FALSE))</f>
         <v>Bitte nutzen Sie zum ausfüllen des Finanzberichts unsere Ausfüllhilfe auf unserer Webseite:</v>
       </c>
@@ -2462,7 +2462,7 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3" spans="2:22">
-      <c r="B3" s="66" t="str">
+      <c r="B3" s="52" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,3,FALSE))</f>
         <v>ÜBERSICHT ÜBER EINNAHMEN UND AUSGABEN</v>
       </c>
@@ -2482,7 +2482,7 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4" spans="2:22" ht="12" customHeight="1">
-      <c r="J4" s="62" t="str">
+      <c r="J4" s="64" t="str">
         <f>HYPERLINK(VLOOKUP($E$2,Sprachversionen!$B:$BN,62,FALSE))</f>
         <v>https://www.kindermissionswerk.org/fuer-partner/service</v>
       </c>
@@ -2572,27 +2572,27 @@
     <row r="11" spans="2:22" ht="12.75" customHeight="1">
       <c r="B11" s="16"/>
       <c r="C11" s="26"/>
-      <c r="D11" s="55" t="str">
+      <c r="D11" s="59" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,11,FALSE))</f>
         <v>Bewilligtes Budget</v>
       </c>
-      <c r="E11" s="63" t="str">
+      <c r="E11" s="66" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,12,FALSE))</f>
         <v>Einnahmen im Berichtszeitraum</v>
       </c>
-      <c r="F11" s="55" t="str">
+      <c r="F11" s="59" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,13,FALSE))</f>
         <v>Einnahmen der gesamten Projektlaufzeit</v>
       </c>
-      <c r="G11" s="55" t="str">
+      <c r="G11" s="59" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,14,FALSE))</f>
         <v>% erhaltene Einnahmen</v>
       </c>
-      <c r="H11" s="67" t="str">
+      <c r="H11" s="60" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,15,FALSE))</f>
         <v>Begründung der Budgetüber- oder unterschreitung</v>
       </c>
-      <c r="J11" s="59" t="str">
+      <c r="J11" s="62" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>KMW Mittel*</v>
       </c>
@@ -2601,7 +2601,7 @@
       <c r="M11" s="34"/>
       <c r="N11" s="34"/>
       <c r="O11" s="35"/>
-      <c r="Q11" s="59" t="str">
+      <c r="Q11" s="62" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>KMW Mittel*</v>
       </c>
@@ -2612,7 +2612,7 @@
       <c r="V11" s="35"/>
     </row>
     <row r="12" spans="2:22">
-      <c r="B12" s="64" t="str">
+      <c r="B12" s="56" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,9,FALSE))</f>
         <v>EINNAHMEN</v>
       </c>
@@ -2636,7 +2636,7 @@
       <c r="V12" s="37"/>
     </row>
     <row r="13" spans="2:22">
-      <c r="B13" s="56" t="str">
+      <c r="B13" s="50" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,10,FALSE))</f>
         <v>(in lokaler Währung)</v>
       </c>
@@ -2660,7 +2660,7 @@
         <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>EUR</v>
       </c>
-      <c r="O13" s="57" t="str">
+      <c r="O13" s="53" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE))</f>
         <v>WK</v>
       </c>
@@ -2678,7 +2678,7 @@
         <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>EUR</v>
       </c>
-      <c r="V13" s="57" t="str">
+      <c r="V13" s="53" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE))</f>
         <v>WK</v>
       </c>
@@ -2721,7 +2721,7 @@
       </c>
     </row>
     <row r="15" spans="2:22">
-      <c r="B15" s="65" t="str">
+      <c r="B15" s="55" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,16,FALSE))</f>
         <v>Saldovortrag (aus vorherigem Berichtszeitraum)</v>
       </c>
@@ -2767,7 +2767,7 @@
       </c>
     </row>
     <row r="16" spans="2:22">
-      <c r="B16" s="50" t="str">
+      <c r="B16" s="58" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,17,FALSE))</f>
         <v>Lokale Eigenleistung</v>
       </c>
@@ -2781,7 +2781,7 @@
       <c r="F16" s="28">
         <v>1000</v>
       </c>
-      <c r="G16" s="52">
+      <c r="G16" s="57">
         <f>IFERROR(F16/D16,0)</f>
         <v>0.5</v>
       </c>
@@ -2816,7 +2816,7 @@
       </c>
     </row>
     <row r="17" spans="2:22">
-      <c r="B17" s="50" t="str">
+      <c r="B17" s="58" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,18,FALSE))</f>
         <v>Beiträge von dritter Seite</v>
       </c>
@@ -2830,7 +2830,7 @@
       <c r="F17" s="28">
         <v>1500</v>
       </c>
-      <c r="G17" s="52">
+      <c r="G17" s="57">
         <f>IFERROR(F17/D17,0)</f>
         <v>0.5</v>
       </c>
@@ -2865,7 +2865,7 @@
       </c>
     </row>
     <row r="18" spans="2:22">
-      <c r="B18" s="50" t="str">
+      <c r="B18" s="58" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>KMW Mittel*</v>
       </c>
@@ -2879,7 +2879,7 @@
       <c r="F18" s="28">
         <v>2000</v>
       </c>
-      <c r="G18" s="52">
+      <c r="G18" s="57">
         <f>IFERROR(F18/D18,0)</f>
         <v>0.5</v>
       </c>
@@ -2914,7 +2914,7 @@
       </c>
     </row>
     <row r="19" spans="2:22">
-      <c r="B19" s="50" t="str">
+      <c r="B19" s="58" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,20,FALSE))</f>
         <v>Zinserträge</v>
       </c>
@@ -2928,7 +2928,7 @@
       <c r="F19" s="28">
         <v>2500</v>
       </c>
-      <c r="G19" s="52">
+      <c r="G19" s="57">
         <f>IFERROR(F19/D19,0)</f>
         <v>0.5</v>
       </c>
@@ -2963,24 +2963,24 @@
       </c>
     </row>
     <row r="20" spans="2:22">
-      <c r="B20" s="61" t="str">
+      <c r="B20" s="51" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,21,FALSE))</f>
         <v>GESAMT</v>
       </c>
       <c r="C20" s="25"/>
-      <c r="D20" s="58">
+      <c r="D20" s="63">
         <f>SUMPRODUCT(ROUND(D15:D19,2))</f>
         <v>15000</v>
       </c>
-      <c r="E20" s="58">
+      <c r="E20" s="63">
         <f>SUMPRODUCT(ROUND(E15:E19,2))</f>
         <v>1500</v>
       </c>
-      <c r="F20" s="58">
+      <c r="F20" s="63">
         <f>SUMPRODUCT(ROUND(F15:F19,2))</f>
         <v>7500</v>
       </c>
-      <c r="G20" s="53">
+      <c r="G20" s="65">
         <f>IFERROR(F20/D20,0)</f>
         <v>0.5</v>
       </c>

</xml_diff>

<commit_message>
Finishing Tests: All right
</commit_message>
<xml_diff>
--- a/src/v2/tests/formula_eval_test.xlsx
+++ b/src/v2/tests/formula_eval_test.xlsx
@@ -2064,57 +2064,57 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -2438,12 +2438,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:22">
-      <c r="B1" s="58" t="str">
+      <c r="B1" s="56" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,2,FALSE))</f>
         <v>F I N A N Z B E R I C H T</v>
       </c>
       <c r="C1" s="3"/>
-      <c r="J1" s="67" t="str">
+      <c r="J1" s="68" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,60,FALSE))</f>
         <v>Tipp:</v>
       </c>
@@ -2458,14 +2458,14 @@
         <v>0</v>
       </c>
       <c r="C2" s="4"/>
-      <c r="D2" s="49" t="str">
+      <c r="D2" s="51" t="str">
         <f>IF($E$2="","Chose your language",VLOOKUP($E$2,Sprachversionen!$B:$BN,27,FALSE))</f>
         <v>Sprache</v>
       </c>
       <c r="E2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="68" t="str">
+      <c r="J2" s="59" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,61,FALSE))</f>
         <v>Bitte nutzen Sie zum ausfüllen des Finanzberichts unsere Ausfüllhilfe auf unserer Webseite:</v>
       </c>
@@ -2476,12 +2476,12 @@
       <c r="O2" s="5"/>
     </row>
     <row r="3" spans="2:22">
-      <c r="B3" s="58" t="str">
+      <c r="B3" s="56" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,3,FALSE))</f>
         <v>ÜBERSICHT ÜBER EINNAHMEN UND AUSGABEN</v>
       </c>
       <c r="C3" s="3"/>
-      <c r="D3" s="49" t="str">
+      <c r="D3" s="51" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE))</f>
         <v>Lokalwährung</v>
       </c>
@@ -2496,7 +2496,7 @@
       <c r="O3" s="5"/>
     </row>
     <row r="4" spans="2:22" ht="12" customHeight="1">
-      <c r="J4" s="64" t="str">
+      <c r="J4" s="65" t="str">
         <f>HYPERLINK(VLOOKUP($E$2,Sprachversionen!$B:$BN,62,FALSE))</f>
         <v>https://www.kindermissionswerk.org/fuer-partner/service</v>
       </c>
@@ -2507,7 +2507,7 @@
       <c r="O4" s="6"/>
     </row>
     <row r="5" spans="2:22">
-      <c r="B5" s="49" t="str">
+      <c r="B5" s="51" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,4,FALSE))</f>
         <v>Projektnummer</v>
       </c>
@@ -2517,7 +2517,7 @@
       </c>
     </row>
     <row r="6" spans="2:22">
-      <c r="B6" s="49" t="str">
+      <c r="B6" s="51" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,26,FALSE))</f>
         <v>Projekttitel</v>
       </c>
@@ -2541,17 +2541,17 @@
       <c r="J7" s="14"/>
     </row>
     <row r="8" spans="2:22">
-      <c r="B8" s="49" t="str">
+      <c r="B8" s="51" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,5,FALSE))</f>
         <v>Projektlaufzeit</v>
       </c>
       <c r="C8" s="7"/>
-      <c r="D8" s="56" t="str">
+      <c r="D8" s="55" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,7,FALSE))</f>
         <v>von (TT MM JJJJ):</v>
       </c>
       <c r="E8" s="9"/>
-      <c r="F8" s="56" t="str">
+      <c r="F8" s="55" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,8,FALSE))</f>
         <v>bis (TT MM JJJJ):</v>
       </c>
@@ -2564,17 +2564,17 @@
       </c>
     </row>
     <row r="9" spans="2:22">
-      <c r="B9" s="49" t="str">
+      <c r="B9" s="51" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,6,FALSE))</f>
         <v>Aktueller Berichtszeitraum</v>
       </c>
       <c r="C9" s="7"/>
-      <c r="D9" s="56" t="str">
+      <c r="D9" s="55" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,7,FALSE))</f>
         <v>von (TT MM JJJJ):</v>
       </c>
       <c r="E9" s="9"/>
-      <c r="F9" s="56" t="str">
+      <c r="F9" s="55" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,8,FALSE))</f>
         <v>bis (TT MM JJJJ):</v>
       </c>
@@ -2586,27 +2586,27 @@
     <row r="11" spans="2:22" ht="12.75" customHeight="1">
       <c r="B11" s="17"/>
       <c r="C11" s="27"/>
-      <c r="D11" s="54" t="str">
+      <c r="D11" s="52" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,11,FALSE))</f>
         <v>Bewilligtes Budget</v>
       </c>
-      <c r="E11" s="53" t="str">
+      <c r="E11" s="57" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,12,FALSE))</f>
         <v>Einnahmen im Berichtszeitraum</v>
       </c>
-      <c r="F11" s="54" t="str">
+      <c r="F11" s="52" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,13,FALSE))</f>
         <v>Einnahmen der gesamten Projektlaufzeit</v>
       </c>
-      <c r="G11" s="54" t="str">
+      <c r="G11" s="52" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,14,FALSE))</f>
         <v>% erhaltene Einnahmen</v>
       </c>
-      <c r="H11" s="65" t="str">
+      <c r="H11" s="63" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,15,FALSE))</f>
         <v>Begründung der Budgetüber- oder unterschreitung</v>
       </c>
-      <c r="J11" s="66" t="str">
+      <c r="J11" s="54" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>KMW Mittel*</v>
       </c>
@@ -2615,7 +2615,7 @@
       <c r="M11" s="35"/>
       <c r="N11" s="35"/>
       <c r="O11" s="36"/>
-      <c r="Q11" s="66" t="str">
+      <c r="Q11" s="54" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>KMW Mittel*</v>
       </c>
@@ -2626,7 +2626,7 @@
       <c r="V11" s="36"/>
     </row>
     <row r="12" spans="2:22">
-      <c r="B12" s="59" t="str">
+      <c r="B12" s="67" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,9,FALSE))</f>
         <v>EINNAHMEN</v>
       </c>
@@ -2650,7 +2650,7 @@
       <c r="V12" s="38"/>
     </row>
     <row r="13" spans="2:22">
-      <c r="B13" s="57" t="str">
+      <c r="B13" s="53" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,10,FALSE))</f>
         <v>(in lokaler Währung)</v>
       </c>
@@ -2674,7 +2674,7 @@
         <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>EUR</v>
       </c>
-      <c r="O13" s="55" t="str">
+      <c r="O13" s="60" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE))</f>
         <v>WK</v>
       </c>
@@ -2692,7 +2692,7 @@
         <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>EUR</v>
       </c>
-      <c r="V13" s="55" t="str">
+      <c r="V13" s="60" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE))</f>
         <v>WK</v>
       </c>
@@ -2735,7 +2735,7 @@
       </c>
     </row>
     <row r="15" spans="2:22">
-      <c r="B15" s="51" t="str">
+      <c r="B15" s="66" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,16,FALSE))</f>
         <v>Saldovortrag (aus vorherigem Berichtszeitraum)</v>
       </c>
@@ -2781,7 +2781,7 @@
       </c>
     </row>
     <row r="16" spans="2:22">
-      <c r="B16" s="61" t="str">
+      <c r="B16" s="64" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,17,FALSE))</f>
         <v>Lokale Eigenleistung</v>
       </c>
@@ -2795,7 +2795,7 @@
       <c r="F16" s="29">
         <v>1000</v>
       </c>
-      <c r="G16" s="52">
+      <c r="G16" s="62">
         <f>IFERROR(F16/D16,0)</f>
         <v>0.5</v>
       </c>
@@ -2830,7 +2830,7 @@
       </c>
     </row>
     <row r="17" spans="2:22">
-      <c r="B17" s="61" t="str">
+      <c r="B17" s="64" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,18,FALSE))</f>
         <v>Beiträge von dritter Seite</v>
       </c>
@@ -2844,7 +2844,7 @@
       <c r="F17" s="29">
         <v>1500</v>
       </c>
-      <c r="G17" s="52">
+      <c r="G17" s="62">
         <f>IFERROR(F17/D17,0)</f>
         <v>0.5</v>
       </c>
@@ -2879,7 +2879,7 @@
       </c>
     </row>
     <row r="18" spans="2:22">
-      <c r="B18" s="61" t="str">
+      <c r="B18" s="64" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>KMW Mittel*</v>
       </c>
@@ -2893,7 +2893,7 @@
       <c r="F18" s="29">
         <v>2000</v>
       </c>
-      <c r="G18" s="52">
+      <c r="G18" s="62">
         <f>IFERROR(F18/D18,0)</f>
         <v>0.5</v>
       </c>
@@ -2928,7 +2928,7 @@
       </c>
     </row>
     <row r="19" spans="2:22">
-      <c r="B19" s="61" t="str">
+      <c r="B19" s="64" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,20,FALSE))</f>
         <v>Zinserträge</v>
       </c>
@@ -2942,7 +2942,7 @@
       <c r="F19" s="29">
         <v>2500</v>
       </c>
-      <c r="G19" s="52">
+      <c r="G19" s="62">
         <f>IFERROR(F19/D19,0)</f>
         <v>0.5</v>
       </c>
@@ -2977,24 +2977,24 @@
       </c>
     </row>
     <row r="20" spans="2:22">
-      <c r="B20" s="63" t="str">
+      <c r="B20" s="58" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,21,FALSE))</f>
         <v>GESAMT</v>
       </c>
       <c r="C20" s="26"/>
-      <c r="D20" s="60">
+      <c r="D20" s="49">
         <f>SUMPRODUCT(ROUND(D15:D19,2))</f>
         <v>15000</v>
       </c>
-      <c r="E20" s="60">
+      <c r="E20" s="49">
         <f>SUMPRODUCT(ROUND(E15:E19,2))</f>
         <v>1500</v>
       </c>
-      <c r="F20" s="60">
+      <c r="F20" s="49">
         <f>SUMPRODUCT(ROUND(F15:F19,2))</f>
         <v>7500</v>
       </c>
-      <c r="G20" s="62">
+      <c r="G20" s="61">
         <f>IFERROR(F20/D20,0)</f>
         <v>0.5</v>
       </c>

</xml_diff>